<commit_message>
Clean notebook: encode raw survey responses, add pinned requirements
</commit_message>
<xml_diff>
--- a/analysis_results.xlsx
+++ b/analysis_results.xlsx
@@ -771,22 +771,22 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>0.5520451375489006</v>
+        <v>0.5520451375489027</v>
       </c>
       <c r="C2" t="n">
         <v>0.1732180889618761</v>
       </c>
       <c r="D2" t="n">
-        <v>3.186994735119156</v>
+        <v>3.186994735119168</v>
       </c>
       <c r="E2" t="n">
-        <v>0.001557869955515148</v>
+        <v>0.001557869955515084</v>
       </c>
       <c r="F2" t="n">
-        <v>0.211447582052007</v>
+        <v>0.2114475820520091</v>
       </c>
       <c r="G2" t="n">
-        <v>0.8926426930457942</v>
+        <v>0.8926426930457962</v>
       </c>
     </row>
     <row r="3">
@@ -796,22 +796,22 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>0.3137563952944</v>
+        <v>0.3137563952944005</v>
       </c>
       <c r="C3" t="n">
-        <v>0.04565776492118422</v>
+        <v>0.04565776492118424</v>
       </c>
       <c r="D3" t="n">
-        <v>6.871917533326818</v>
+        <v>6.871917533326827</v>
       </c>
       <c r="E3" t="n">
-        <v>2.641175618307216e-11</v>
+        <v>2.641175618307081e-11</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2239798412704736</v>
+        <v>0.223979841270474</v>
       </c>
       <c r="G3" t="n">
-        <v>0.4035329493183265</v>
+        <v>0.403532949318327</v>
       </c>
     </row>
     <row r="4">
@@ -821,22 +821,22 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>0.2409541893213112</v>
+        <v>0.2409541893213104</v>
       </c>
       <c r="C4" t="n">
-        <v>0.05048441242050353</v>
+        <v>0.05048441242050355</v>
       </c>
       <c r="D4" t="n">
-        <v>4.772843294962289</v>
+        <v>4.772843294962272</v>
       </c>
       <c r="E4" t="n">
-        <v>2.605162866776078e-06</v>
+        <v>2.605162866776278e-06</v>
       </c>
       <c r="F4" t="n">
-        <v>0.1416870309998441</v>
+        <v>0.1416870309998433</v>
       </c>
       <c r="G4" t="n">
-        <v>0.3402213476427782</v>
+        <v>0.3402213476427774</v>
       </c>
     </row>
     <row r="5">
@@ -846,22 +846,22 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>0.4046187836602092</v>
+        <v>0.4046187836602094</v>
       </c>
       <c r="C5" t="n">
         <v>0.04435170851168052</v>
       </c>
       <c r="D5" t="n">
-        <v>9.122958218253267</v>
+        <v>9.122958218253272</v>
       </c>
       <c r="E5" t="n">
-        <v>4.506188401678489e-18</v>
+        <v>4.506188401678341e-18</v>
       </c>
       <c r="F5" t="n">
-        <v>0.3174103195112145</v>
+        <v>0.3174103195112146</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4918272478092039</v>
+        <v>0.4918272478092041</v>
       </c>
     </row>
   </sheetData>
@@ -1089,10 +1089,10 @@
         <v>0.309</v>
       </c>
       <c r="F2" t="n">
-        <v>0.05693816319265893</v>
+        <v>0.05693816257934232</v>
       </c>
       <c r="G2" t="n">
-        <v>4.94450108315529</v>
+        <v>4.94450124553039</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1121,10 +1121,10 @@
         <v>0.188</v>
       </c>
       <c r="F3" t="n">
-        <v>0.06289419867465651</v>
+        <v>0.06289419652572176</v>
       </c>
       <c r="G3" t="n">
-        <v>3.739785826584722</v>
+        <v>3.739785834265285</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -1153,10 +1153,10 @@
         <v>0.447</v>
       </c>
       <c r="F4" t="n">
-        <v>0.06029511169803593</v>
+        <v>0.06029511217919249</v>
       </c>
       <c r="G4" t="n">
-        <v>7.584174772014924</v>
+        <v>7.584175059517517</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -1219,10 +1219,10 @@
         <v>0.881</v>
       </c>
       <c r="F6" t="n">
-        <v>0.04545656614497126</v>
+        <v>0.04545656496501785</v>
       </c>
       <c r="G6" t="n">
-        <v>23.15171521643995</v>
+        <v>23.15171592605234</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -1251,10 +1251,10 @@
         <v>0.824</v>
       </c>
       <c r="F7" t="n">
-        <v>0.04535666715024489</v>
+        <v>0.0453566663186009</v>
       </c>
       <c r="G7" t="n">
-        <v>20.54792476302647</v>
+        <v>20.54792542011821</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -1283,10 +1283,10 @@
         <v>0.863</v>
       </c>
       <c r="F8" t="n">
-        <v>0.04450155891523704</v>
+        <v>0.04450155734808903</v>
       </c>
       <c r="G8" t="n">
-        <v>22.30242796703018</v>
+        <v>22.30242824937984</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -1315,10 +1315,10 @@
         <v>0.8149999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>0.04524402563440771</v>
+        <v>0.04524402398005042</v>
       </c>
       <c r="G9" t="n">
-        <v>20.16890704704405</v>
+        <v>20.16890734055633</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -1381,10 +1381,10 @@
         <v>0.871</v>
       </c>
       <c r="F11" t="n">
-        <v>0.05350168622067793</v>
+        <v>0.05350168167144796</v>
       </c>
       <c r="G11" t="n">
-        <v>20.86719292651416</v>
+        <v>20.8671942835649</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1413,10 +1413,10 @@
         <v>0.827</v>
       </c>
       <c r="F12" t="n">
-        <v>0.05356377716544965</v>
+        <v>0.05356377399878681</v>
       </c>
       <c r="G12" t="n">
-        <v>19.24729307690981</v>
+        <v>19.24729399968962</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -1445,10 +1445,10 @@
         <v>0.796</v>
       </c>
       <c r="F13" t="n">
-        <v>0.05757217757502306</v>
+        <v>0.05757217297514181</v>
       </c>
       <c r="G13" t="n">
-        <v>18.21201527073729</v>
+        <v>18.21201593321404</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -1477,10 +1477,10 @@
         <v>0.867</v>
       </c>
       <c r="F14" t="n">
-        <v>0.05461708865675959</v>
+        <v>0.05461708484579232</v>
       </c>
       <c r="G14" t="n">
-        <v>20.72410572762766</v>
+        <v>20.72410719008202</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -1543,10 +1543,10 @@
         <v>0.821</v>
       </c>
       <c r="F16" t="n">
-        <v>0.05704702468663512</v>
+        <v>0.05704702624903303</v>
       </c>
       <c r="G16" t="n">
-        <v>18.08566839145888</v>
+        <v>18.08566829486005</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1575,10 +1575,10 @@
         <v>0.8120000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0592886631795992</v>
+        <v>0.0592886623344844</v>
       </c>
       <c r="G17" t="n">
-        <v>17.83150446138352</v>
+        <v>17.83150424464268</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1607,10 +1607,10 @@
         <v>0.793</v>
       </c>
       <c r="F18" t="n">
-        <v>0.05743463192383533</v>
+        <v>0.05743463187413503</v>
       </c>
       <c r="G18" t="n">
-        <v>17.24970592550032</v>
+        <v>17.24970609959675</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1639,10 +1639,10 @@
         <v>0.78</v>
       </c>
       <c r="F19" t="n">
-        <v>0.05793812338678674</v>
+        <v>0.05793812358334258</v>
       </c>
       <c r="G19" t="n">
-        <v>16.87992374361337</v>
+        <v>16.87992340837948</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -1705,10 +1705,10 @@
         <v>0.855</v>
       </c>
       <c r="F21" t="n">
-        <v>0.05443697131762475</v>
+        <v>0.05443696907976063</v>
       </c>
       <c r="G21" t="n">
-        <v>19.23670303014974</v>
+        <v>19.23670358304008</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1737,10 +1737,10 @@
         <v>0.797</v>
       </c>
       <c r="F22" t="n">
-        <v>0.05640644487444762</v>
+        <v>0.0564064426638854</v>
       </c>
       <c r="G22" t="n">
-        <v>17.47210040557678</v>
+        <v>17.47210102792041</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1769,10 +1769,10 @@
         <v>0.848</v>
       </c>
       <c r="F23" t="n">
-        <v>0.05607214076844908</v>
+        <v>0.05607213831842262</v>
       </c>
       <c r="G23" t="n">
-        <v>19.04161598135293</v>
+        <v>19.04161674597673</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1801,10 +1801,10 @@
         <v>0.857</v>
       </c>
       <c r="F24" t="n">
-        <v>0.05632944187818699</v>
+        <v>0.05632944046792585</v>
       </c>
       <c r="G24" t="n">
-        <v>19.3123090561118</v>
+        <v>19.31231006386775</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1833,10 +1833,10 @@
         <v>0.306</v>
       </c>
       <c r="F25" t="n">
-        <v>0.007170815602308834</v>
+        <v>0.007170815451199838</v>
       </c>
       <c r="G25" t="n">
-        <v>7.990649614044763</v>
+        <v>7.990649676928316</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1865,10 +1865,10 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>0.02174166525897996</v>
+        <v>0.02174166610737093</v>
       </c>
       <c r="G26" t="n">
-        <v>10.39492951721432</v>
+        <v>10.39492967367515</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1897,10 +1897,10 @@
         <v>0.706</v>
       </c>
       <c r="F27" t="n">
-        <v>0.01487385781463312</v>
+        <v>0.01487385830538044</v>
       </c>
       <c r="G27" t="n">
-        <v>9.546716007767847</v>
+        <v>9.546716090345829</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1929,10 +1929,10 @@
         <v>1</v>
       </c>
       <c r="F28" t="n">
-        <v>0.01920477193466053</v>
+        <v>0.01920477213198376</v>
       </c>
       <c r="G28" t="n">
-        <v>9.312398168472239</v>
+        <v>9.312398175653867</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -1961,10 +1961,10 @@
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>0.01232589730561466</v>
+        <v>0.01232589789628216</v>
       </c>
       <c r="G29" t="n">
-        <v>9.724514700441828</v>
+        <v>9.724515112937851</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -1993,10 +1993,10 @@
         <v>0.664</v>
       </c>
       <c r="F30" t="n">
-        <v>0.01170529379713988</v>
+        <v>0.01170529457604096</v>
       </c>
       <c r="G30" t="n">
-        <v>9.342412563686903</v>
+        <v>9.34241281721089</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -2025,10 +2025,10 @@
         <v>0.546</v>
       </c>
       <c r="F31" t="n">
-        <v>0.00997953546303704</v>
+        <v>0.009979535952052287</v>
       </c>
       <c r="G31" t="n">
-        <v>8.009191848819651</v>
+        <v>8.009192024930346</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -2057,10 +2057,10 @@
         <v>0.358</v>
       </c>
       <c r="F32" t="n">
-        <v>0.008751333337335052</v>
+        <v>0.008751333246577757</v>
       </c>
       <c r="G32" t="n">
-        <v>11.93217037435583</v>
+        <v>11.93217038166475</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -2089,10 +2089,10 @@
         <v>0.27</v>
       </c>
       <c r="F33" t="n">
-        <v>0.006913883172657107</v>
+        <v>0.006913883231875728</v>
       </c>
       <c r="G33" t="n">
-        <v>10.97173770033683</v>
+        <v>10.97173788044834</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -2121,10 +2121,10 @@
         <v>0.365</v>
       </c>
       <c r="F34" t="n">
-        <v>0.008731604808959331</v>
+        <v>0.008731604775688732</v>
       </c>
       <c r="G34" t="n">
-        <v>11.9909305086677</v>
+        <v>11.99093054506868</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -2153,10 +2153,10 @@
         <v>0.28</v>
       </c>
       <c r="F35" t="n">
-        <v>0.007480213154392366</v>
+        <v>0.007480213012875287</v>
       </c>
       <c r="G35" t="n">
-        <v>11.11943848610697</v>
+        <v>11.11943849247972</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -2185,10 +2185,10 @@
         <v>0.265</v>
       </c>
       <c r="F36" t="n">
-        <v>0.007346329046575358</v>
+        <v>0.007346329008844981</v>
       </c>
       <c r="G36" t="n">
-        <v>10.91127439729291</v>
+        <v>10.91127421624955</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -2217,10 +2217,10 @@
         <v>0.257</v>
       </c>
       <c r="F37" t="n">
-        <v>0.007065034126390165</v>
+        <v>0.007065034086791528</v>
       </c>
       <c r="G37" t="n">
-        <v>11.07825700923446</v>
+        <v>11.07825691744291</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -2249,10 +2249,10 @@
         <v>0.225</v>
       </c>
       <c r="F38" t="n">
-        <v>0.006877065970973172</v>
+        <v>0.006877066098660144</v>
       </c>
       <c r="G38" t="n">
-        <v>10.54377407753498</v>
+        <v>10.54377402891646</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -2281,10 +2281,10 @@
         <v>0.321</v>
       </c>
       <c r="F39" t="n">
-        <v>0.007855093587567663</v>
+        <v>0.007855093803631528</v>
       </c>
       <c r="G39" t="n">
-        <v>11.81136435089892</v>
+        <v>11.81136430426251</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -2313,10 +2313,10 @@
         <v>0.255</v>
       </c>
       <c r="F40" t="n">
-        <v>0.006909019781500172</v>
+        <v>0.006909019919277087</v>
       </c>
       <c r="G40" t="n">
-        <v>11.0515863943024</v>
+        <v>11.05158656262285</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -2345,10 +2345,10 @@
         <v>0.336</v>
       </c>
       <c r="F41" t="n">
-        <v>0.007959087106883788</v>
+        <v>0.007959087163597174</v>
       </c>
       <c r="G41" t="n">
-        <v>11.93955848529382</v>
+        <v>11.93955855550579</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -2377,10 +2377,10 @@
         <v>0.345</v>
       </c>
       <c r="F42" t="n">
-        <v>0.008354902419644742</v>
+        <v>0.008354902500403867</v>
       </c>
       <c r="G42" t="n">
-        <v>11.28094784772319</v>
+        <v>11.28094781271627</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -2409,10 +2409,10 @@
         <v>0.326</v>
       </c>
       <c r="F43" t="n">
-        <v>0.008328374476686183</v>
+        <v>0.008328375109770291</v>
       </c>
       <c r="G43" t="n">
-        <v>11.05312446146617</v>
+        <v>11.05312450405984</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -2441,10 +2441,10 @@
         <v>0.34</v>
       </c>
       <c r="F44" t="n">
-        <v>0.009173530334211945</v>
+        <v>0.009173530348144455</v>
       </c>
       <c r="G44" t="n">
-        <v>11.22184117946508</v>
+        <v>11.22184129415335</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -2473,10 +2473,10 @@
         <v>0.372</v>
       </c>
       <c r="F45" t="n">
-        <v>0.008986845845362119</v>
+        <v>0.008986845836175761</v>
       </c>
       <c r="G45" t="n">
-        <v>11.55832432807974</v>
+        <v>11.55832421622793</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -2505,10 +2505,10 @@
         <v>0.392</v>
       </c>
       <c r="F46" t="n">
-        <v>0.009386248553447702</v>
+        <v>0.009386248956335006</v>
       </c>
       <c r="G46" t="n">
-        <v>11.74256655344468</v>
+        <v>11.74256669285792</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -2537,10 +2537,10 @@
         <v>0.314</v>
       </c>
       <c r="F47" t="n">
-        <v>0.004791710056925315</v>
+        <v>0.004791709791853065</v>
       </c>
       <c r="G47" t="n">
-        <v>11.44053499350689</v>
+        <v>11.44053477002164</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -2569,10 +2569,10 @@
         <v>0.241</v>
       </c>
       <c r="F48" t="n">
-        <v>0.004562327781644086</v>
+        <v>0.004562327696248147</v>
       </c>
       <c r="G48" t="n">
-        <v>10.38588772118397</v>
+        <v>10.38588773297569</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -2601,10 +2601,10 @@
         <v>0.317</v>
       </c>
       <c r="F49" t="n">
-        <v>0.005149111793195341</v>
+        <v>0.005149112007235683</v>
       </c>
       <c r="G49" t="n">
-        <v>11.47332889092318</v>
+        <v>11.47332902503648</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -2633,10 +2633,10 @@
         <v>0.366</v>
       </c>
       <c r="F50" t="n">
-        <v>0.006367244892764035</v>
+        <v>0.006367244911784253</v>
       </c>
       <c r="G50" t="n">
-        <v>11.93322986292756</v>
+        <v>11.93323002261393</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -2665,10 +2665,10 @@
         <v>0.248</v>
       </c>
       <c r="F51" t="n">
-        <v>0.004807399796690094</v>
+        <v>0.004807399804144202</v>
       </c>
       <c r="G51" t="n">
-        <v>10.50828816348452</v>
+        <v>10.50828807247138</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Add R robustness notebook and extended N = 380 analyses
</commit_message>
<xml_diff>
--- a/analysis_results.xlsx
+++ b/analysis_results.xlsx
@@ -1089,10 +1089,10 @@
         <v>0.309</v>
       </c>
       <c r="F2" t="n">
-        <v>0.05693816257934232</v>
+        <v>0.05693816243111144</v>
       </c>
       <c r="G2" t="n">
-        <v>4.94450124553039</v>
+        <v>4.944501282202579</v>
       </c>
       <c r="H2" t="n">
         <v>0</v>
@@ -1121,10 +1121,10 @@
         <v>0.188</v>
       </c>
       <c r="F3" t="n">
-        <v>0.06289419652572176</v>
+        <v>0.0628941960186685</v>
       </c>
       <c r="G3" t="n">
-        <v>3.739785834265285</v>
+        <v>3.739785839705894</v>
       </c>
       <c r="H3" t="n">
         <v>0</v>
@@ -1153,10 +1153,10 @@
         <v>0.447</v>
       </c>
       <c r="F4" t="n">
-        <v>0.06029511217919249</v>
+        <v>0.06029511230316668</v>
       </c>
       <c r="G4" t="n">
-        <v>7.584175059517517</v>
+        <v>7.584175120048824</v>
       </c>
       <c r="H4" t="n">
         <v>0</v>
@@ -1219,10 +1219,10 @@
         <v>0.881</v>
       </c>
       <c r="F6" t="n">
-        <v>0.04545656496501785</v>
+        <v>0.04545656472029785</v>
       </c>
       <c r="G6" t="n">
-        <v>23.15171592605234</v>
+        <v>23.15171608334466</v>
       </c>
       <c r="H6" t="n">
         <v>0</v>
@@ -1251,10 +1251,10 @@
         <v>0.824</v>
       </c>
       <c r="F7" t="n">
-        <v>0.0453566663186009</v>
+        <v>0.04535666614952556</v>
       </c>
       <c r="G7" t="n">
-        <v>20.54792542011821</v>
+        <v>20.54792556986881</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -1283,10 +1283,10 @@
         <v>0.863</v>
       </c>
       <c r="F8" t="n">
-        <v>0.04450155734808903</v>
+        <v>0.04450155702150089</v>
       </c>
       <c r="G8" t="n">
-        <v>22.30242824937984</v>
+        <v>22.30242831816859</v>
       </c>
       <c r="H8" t="n">
         <v>0</v>
@@ -1315,10 +1315,10 @@
         <v>0.8149999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>0.04524402398005042</v>
+        <v>0.04524402360974235</v>
       </c>
       <c r="G9" t="n">
-        <v>20.16890734055633</v>
+        <v>20.16890739322275</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -1381,10 +1381,10 @@
         <v>0.871</v>
       </c>
       <c r="F11" t="n">
-        <v>0.05350168167144796</v>
+        <v>0.05350168064424733</v>
       </c>
       <c r="G11" t="n">
-        <v>20.8671942835649</v>
+        <v>20.86719458785957</v>
       </c>
       <c r="H11" t="n">
         <v>0</v>
@@ -1413,10 +1413,10 @@
         <v>0.827</v>
       </c>
       <c r="F12" t="n">
-        <v>0.05356377399878681</v>
+        <v>0.05356377328467132</v>
       </c>
       <c r="G12" t="n">
-        <v>19.24729399968962</v>
+        <v>19.24729420979249</v>
       </c>
       <c r="H12" t="n">
         <v>0</v>
@@ -1445,10 +1445,10 @@
         <v>0.796</v>
       </c>
       <c r="F13" t="n">
-        <v>0.05757217297514181</v>
+        <v>0.05757217192338567</v>
       </c>
       <c r="G13" t="n">
-        <v>18.21201593321404</v>
+        <v>18.21201608011926</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -1477,10 +1477,10 @@
         <v>0.867</v>
       </c>
       <c r="F14" t="n">
-        <v>0.05461708484579232</v>
+        <v>0.05461708397692035</v>
       </c>
       <c r="G14" t="n">
-        <v>20.72410719008202</v>
+        <v>20.72410751904829</v>
       </c>
       <c r="H14" t="n">
         <v>0</v>
@@ -1543,10 +1543,10 @@
         <v>0.821</v>
       </c>
       <c r="F16" t="n">
-        <v>0.05704702624903303</v>
+        <v>0.05704702664887444</v>
       </c>
       <c r="G16" t="n">
-        <v>18.08566829486005</v>
+        <v>18.0856682653623</v>
       </c>
       <c r="H16" t="n">
         <v>0</v>
@@ -1575,10 +1575,10 @@
         <v>0.8120000000000001</v>
       </c>
       <c r="F17" t="n">
-        <v>0.0592886623344844</v>
+        <v>0.0592886621967198</v>
       </c>
       <c r="G17" t="n">
-        <v>17.83150424464268</v>
+        <v>17.83150418702712</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -1607,10 +1607,10 @@
         <v>0.793</v>
       </c>
       <c r="F18" t="n">
-        <v>0.05743463187413503</v>
+        <v>0.05743463190667211</v>
       </c>
       <c r="G18" t="n">
-        <v>17.24970609959675</v>
+        <v>17.24970612861383</v>
       </c>
       <c r="H18" t="n">
         <v>0</v>
@@ -1639,10 +1639,10 @@
         <v>0.78</v>
       </c>
       <c r="F19" t="n">
-        <v>0.05793812358334258</v>
+        <v>0.05793812366591149</v>
       </c>
       <c r="G19" t="n">
-        <v>16.87992340837948</v>
+        <v>16.87992331953979</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -1705,10 +1705,10 @@
         <v>0.855</v>
       </c>
       <c r="F21" t="n">
-        <v>0.05443696907976063</v>
+        <v>0.05443696861045999</v>
       </c>
       <c r="G21" t="n">
-        <v>19.23670358304008</v>
+        <v>19.23670369942031</v>
       </c>
       <c r="H21" t="n">
         <v>0</v>
@@ -1737,10 +1737,10 @@
         <v>0.797</v>
       </c>
       <c r="F22" t="n">
-        <v>0.0564064426638854</v>
+        <v>0.05640644219171657</v>
       </c>
       <c r="G22" t="n">
-        <v>17.47210102792041</v>
+        <v>17.47210116029856</v>
       </c>
       <c r="H22" t="n">
         <v>0</v>
@@ -1769,10 +1769,10 @@
         <v>0.848</v>
       </c>
       <c r="F23" t="n">
-        <v>0.05607213831842262</v>
+        <v>0.05607213779742307</v>
       </c>
       <c r="G23" t="n">
-        <v>19.04161674597673</v>
+        <v>19.04161690639226</v>
       </c>
       <c r="H23" t="n">
         <v>0</v>
@@ -1801,10 +1801,10 @@
         <v>0.857</v>
       </c>
       <c r="F24" t="n">
-        <v>0.05632944046792585</v>
+        <v>0.05632944018042869</v>
       </c>
       <c r="G24" t="n">
-        <v>19.31231006386775</v>
+        <v>19.31231027855744</v>
       </c>
       <c r="H24" t="n">
         <v>0</v>
@@ -1833,10 +1833,10 @@
         <v>0.306</v>
       </c>
       <c r="F25" t="n">
-        <v>0.007170815451199838</v>
+        <v>0.007170815413832618</v>
       </c>
       <c r="G25" t="n">
-        <v>7.990649676928316</v>
+        <v>7.99064968882669</v>
       </c>
       <c r="H25" t="n">
         <v>0</v>
@@ -1865,10 +1865,10 @@
         <v>1</v>
       </c>
       <c r="F26" t="n">
-        <v>0.02174166610737093</v>
+        <v>0.02174166629384445</v>
       </c>
       <c r="G26" t="n">
-        <v>10.39492967367515</v>
+        <v>10.39492970717162</v>
       </c>
       <c r="H26" t="n">
         <v>0</v>
@@ -1897,10 +1897,10 @@
         <v>0.706</v>
       </c>
       <c r="F27" t="n">
-        <v>0.01487385830538044</v>
+        <v>0.0148738584046952</v>
       </c>
       <c r="G27" t="n">
-        <v>9.546716090345829</v>
+        <v>9.546716106860513</v>
       </c>
       <c r="H27" t="n">
         <v>0</v>
@@ -1909,7 +1909,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>income_expect</t>
+          <t>employability</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1919,20 +1919,20 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>income_expect</t>
+          <t>skill_relevance</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.179</v>
+        <v>0.109</v>
       </c>
       <c r="E28" t="n">
-        <v>1</v>
+        <v>0.664</v>
       </c>
       <c r="F28" t="n">
-        <v>0.01920477213198376</v>
+        <v>0.0117052947484398</v>
       </c>
       <c r="G28" t="n">
-        <v>9.312398175653867</v>
+        <v>9.34241287337777</v>
       </c>
       <c r="H28" t="n">
         <v>0</v>
@@ -1941,7 +1941,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>skill_relevance</t>
+          <t>income_expect</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1951,20 +1951,20 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>skill_relevance</t>
+          <t>income_expect</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.12</v>
+        <v>0.179</v>
       </c>
       <c r="E29" t="n">
         <v>1</v>
       </c>
       <c r="F29" t="n">
-        <v>0.01232589789628216</v>
+        <v>0.01920477215855214</v>
       </c>
       <c r="G29" t="n">
-        <v>9.724515112937851</v>
+        <v>9.312398173682896</v>
       </c>
       <c r="H29" t="n">
         <v>0</v>
@@ -1983,20 +1983,20 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>employability</t>
+          <t>skill_relevance</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.109</v>
+        <v>0.12</v>
       </c>
       <c r="E30" t="n">
-        <v>0.664</v>
+        <v>1</v>
       </c>
       <c r="F30" t="n">
-        <v>0.01170529457604096</v>
+        <v>0.01232589802749195</v>
       </c>
       <c r="G30" t="n">
-        <v>9.34241281721089</v>
+        <v>9.724515206715074</v>
       </c>
       <c r="H30" t="n">
         <v>0</v>
@@ -2025,10 +2025,10 @@
         <v>0.546</v>
       </c>
       <c r="F31" t="n">
-        <v>0.009979535952052287</v>
+        <v>0.009979536054864556</v>
       </c>
       <c r="G31" t="n">
-        <v>8.009192024930346</v>
+        <v>8.009192061768246</v>
       </c>
       <c r="H31" t="n">
         <v>0</v>
@@ -2057,10 +2057,10 @@
         <v>0.358</v>
       </c>
       <c r="F32" t="n">
-        <v>0.008751333246577757</v>
+        <v>0.008751333225679383</v>
       </c>
       <c r="G32" t="n">
-        <v>11.93217038166475</v>
+        <v>11.9321703832145</v>
       </c>
       <c r="H32" t="n">
         <v>0</v>
@@ -2089,10 +2089,10 @@
         <v>0.27</v>
       </c>
       <c r="F33" t="n">
-        <v>0.006913883231875728</v>
+        <v>0.006913883245613727</v>
       </c>
       <c r="G33" t="n">
-        <v>10.97173788044834</v>
+        <v>10.971737919632</v>
       </c>
       <c r="H33" t="n">
         <v>0</v>
@@ -2121,10 +2121,10 @@
         <v>0.365</v>
       </c>
       <c r="F34" t="n">
-        <v>0.008731604775688732</v>
+        <v>0.008731604766240245</v>
       </c>
       <c r="G34" t="n">
-        <v>11.99093054506868</v>
+        <v>11.99093055276383</v>
       </c>
       <c r="H34" t="n">
         <v>0</v>
@@ -2153,10 +2153,10 @@
         <v>0.28</v>
       </c>
       <c r="F35" t="n">
-        <v>0.007480213012875287</v>
+        <v>0.007480212982929856</v>
       </c>
       <c r="G35" t="n">
-        <v>11.11943849247972</v>
+        <v>11.11943849537156</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -2185,10 +2185,10 @@
         <v>0.265</v>
       </c>
       <c r="F36" t="n">
-        <v>0.007346329008844981</v>
+        <v>0.007346329002316006</v>
       </c>
       <c r="G36" t="n">
-        <v>10.91127421624955</v>
+        <v>10.91127417737645</v>
       </c>
       <c r="H36" t="n">
         <v>0</v>
@@ -2217,10 +2217,10 @@
         <v>0.257</v>
       </c>
       <c r="F37" t="n">
-        <v>0.007065034086791528</v>
+        <v>0.007065034079339046</v>
       </c>
       <c r="G37" t="n">
-        <v>11.07825691744291</v>
+        <v>11.07825689935718</v>
       </c>
       <c r="H37" t="n">
         <v>0</v>
@@ -2249,10 +2249,10 @@
         <v>0.225</v>
       </c>
       <c r="F38" t="n">
-        <v>0.006877066098660144</v>
+        <v>0.006877066127433429</v>
       </c>
       <c r="G38" t="n">
-        <v>10.54377402891646</v>
+        <v>10.5437740169989</v>
       </c>
       <c r="H38" t="n">
         <v>0</v>
@@ -2281,10 +2281,10 @@
         <v>0.321</v>
       </c>
       <c r="F39" t="n">
-        <v>0.007855093803631528</v>
+        <v>0.007855093851124997</v>
       </c>
       <c r="G39" t="n">
-        <v>11.81136430426251</v>
+        <v>11.81136429226471</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
@@ -2313,10 +2313,10 @@
         <v>0.255</v>
       </c>
       <c r="F40" t="n">
-        <v>0.006909019919277087</v>
+        <v>0.006909019949656913</v>
       </c>
       <c r="G40" t="n">
-        <v>11.05158656262285</v>
+        <v>11.05158659593145</v>
       </c>
       <c r="H40" t="n">
         <v>0</v>
@@ -2345,10 +2345,10 @@
         <v>0.336</v>
       </c>
       <c r="F41" t="n">
-        <v>0.007959087163597174</v>
+        <v>0.007959087175518593</v>
       </c>
       <c r="G41" t="n">
-        <v>11.93955855550579</v>
+        <v>11.93955857493893</v>
       </c>
       <c r="H41" t="n">
         <v>0</v>
@@ -2377,10 +2377,10 @@
         <v>0.345</v>
       </c>
       <c r="F42" t="n">
-        <v>0.008354902500403867</v>
+        <v>0.008354902517865437</v>
       </c>
       <c r="G42" t="n">
-        <v>11.28094781271627</v>
+        <v>11.28094780611273</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
@@ -2409,10 +2409,10 @@
         <v>0.326</v>
       </c>
       <c r="F43" t="n">
-        <v>0.008328375109770291</v>
+        <v>0.008328375250507775</v>
       </c>
       <c r="G43" t="n">
-        <v>11.05312450405984</v>
+        <v>11.05312451155986</v>
       </c>
       <c r="H43" t="n">
         <v>0</v>
@@ -2441,10 +2441,10 @@
         <v>0.34</v>
       </c>
       <c r="F44" t="n">
-        <v>0.009173530348144455</v>
+        <v>0.009173530351119088</v>
       </c>
       <c r="G44" t="n">
-        <v>11.22184129415335</v>
+        <v>11.22184131888389</v>
       </c>
       <c r="H44" t="n">
         <v>0</v>
@@ -2473,10 +2473,10 @@
         <v>0.372</v>
       </c>
       <c r="F45" t="n">
-        <v>0.008986845836175761</v>
+        <v>0.008986845833145874</v>
       </c>
       <c r="G45" t="n">
-        <v>11.55832421622793</v>
+        <v>11.55832419112379</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
@@ -2505,10 +2505,10 @@
         <v>0.392</v>
       </c>
       <c r="F46" t="n">
-        <v>0.009386248956335006</v>
+        <v>0.009386249046525691</v>
       </c>
       <c r="G46" t="n">
-        <v>11.74256669285792</v>
+        <v>11.74256672596404</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
@@ -2537,10 +2537,10 @@
         <v>0.314</v>
       </c>
       <c r="F47" t="n">
-        <v>0.004791709791853065</v>
+        <v>0.004791709730638962</v>
       </c>
       <c r="G47" t="n">
-        <v>11.44053477002164</v>
+        <v>11.44053471792785</v>
       </c>
       <c r="H47" t="n">
         <v>0</v>
@@ -2569,10 +2569,10 @@
         <v>0.241</v>
       </c>
       <c r="F48" t="n">
-        <v>0.004562327696248147</v>
+        <v>0.004562327678624531</v>
       </c>
       <c r="G48" t="n">
-        <v>10.38588773297569</v>
+        <v>10.38588773723561</v>
       </c>
       <c r="H48" t="n">
         <v>0</v>
@@ -2601,10 +2601,10 @@
         <v>0.317</v>
       </c>
       <c r="F49" t="n">
-        <v>0.005149112007235683</v>
+        <v>0.0051491120557376</v>
       </c>
       <c r="G49" t="n">
-        <v>11.47332902503648</v>
+        <v>11.47332905402155</v>
       </c>
       <c r="H49" t="n">
         <v>0</v>
@@ -2633,10 +2633,10 @@
         <v>0.366</v>
       </c>
       <c r="F50" t="n">
-        <v>0.006367244911784253</v>
+        <v>0.006367244914738439</v>
       </c>
       <c r="G50" t="n">
-        <v>11.93323002261393</v>
+        <v>11.93323005930066</v>
       </c>
       <c r="H50" t="n">
         <v>0</v>
@@ -2665,10 +2665,10 @@
         <v>0.248</v>
       </c>
       <c r="F51" t="n">
-        <v>0.004807399804144202</v>
+        <v>0.004807399805735232</v>
       </c>
       <c r="G51" t="n">
-        <v>10.50828807247138</v>
+        <v>10.50828805267044</v>
       </c>
       <c r="H51" t="n">
         <v>0</v>

</xml_diff>